<commit_message>
Record verified Kickoff enrollment trigger from WLS screenshot
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TuFPqtNuPi7KBKeykeDCDb
</commit_message>
<xml_diff>
--- a/audits/transitions-workflow-audit/WLS_Transitions_Workflow_Audit.xlsx
+++ b/audits/transitions-workflow-audit/WLS_Transitions_Workflow_Audit.xlsx
@@ -524,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A37"/>
+  <dimension ref="A1:A38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -588,167 +588,174 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>VERIFIED (records) - directly visible in HubSpot task / ticket / deal records. Not the workflow configuration itself.</t>
+          <t>VERIFIED (screenshot) - workflow configuration seen in a screenshot of the HubSpot workflow editor supplied by WLS. This is real configuration.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>INFERENCE - logically derived from the records (for example: tasks appear within seconds of a ticket entering a stage, so the trigger is probably "ticket enters stage"). Not proven.</t>
+          <t>VERIFIED (records) - directly visible in HubSpot task / ticket / deal records. Not the workflow configuration itself.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>INFERENCE - logically derived from the records (for example: tasks appear within seconds of a ticket entering a stage, so the trigger is probably "ticket enters stage"). Not proven.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
           <t>NEEDS VERIFICATION - cannot be determined without opening the workflow in HubSpot.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr"/>
-    </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>HOW TO READ "ACTION #"</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Action # = HubSpot's actionExecutionIndex + 1, taken from each task's Record creation source ID. It is the order in which the enrollment executed actions. It is NOT necessarily the step number shown in the workflow editor: branches, delays and property edits that create no task leave no record. A gap in the sequence (e.g. Pre-Launch #6-#7) means something ran there that created no task.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
-    </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>DUE DATES, OWNERS, TITLES</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Values are the CURRENT values on each task. Users may have edited due dates, owners or titles after creation, so the most common value (shown with its count, e.g. 18/21) is the best evidence of what the workflow sets. Times are US/Eastern (portal time zone). "bd" = business days (Mon-Fri) between creation date and due date.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr"/>
-    </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>SCOPE - these 8 workflows only</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>1. Closed Won | Create Ticket in INITIAL SETUP - UNASSIGNED (ID 1670039203) - creates the ticket.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2. Transitions - Transition Kickoff Tasks (+SubTask)</t>
+          <t>1. Closed Won | Create Ticket in INITIAL SETUP - UNASSIGNED (ID 1670039203) - creates the ticket.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>3. Transitions - Pre Launch Setup Tasks (+SubTask)</t>
+          <t>2. Transitions - Transition Kickoff Tasks (+SubTask)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>4. Transitions - Launch Readiness Tasks (+SubTask)</t>
+          <t>3. Transitions - Pre Launch Setup Tasks (+SubTask)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>5. Transitions - Go Live Execution Tasks (+SubTask)</t>
+          <t>4. Transitions - Launch Readiness Tasks (+SubTask)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>6. Transitions - Final Sign Off Tasks (+SubTask)</t>
+          <t>5. Transitions - Go Live Execution Tasks (+SubTask)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>7. Transitions - 30-Day Monitoring (+SubTask)</t>
+          <t>6. Transitions - Final Sign Off Tasks (+SubTask)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>8. Transitions - TRANSITION COMPLETE (+SubTask)</t>
+          <t>7. Transitions - 30-Day Monitoring (+SubTask)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
+          <t>8. Transitions - TRANSITION COMPLETE (+SubTask)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
           <t>Other workflows (legacy non-subtask versions, Set task queue, Set OM and SM overdue tasks to Deferred, Marketing Proposal Task) are mentioned only in Audit Findings, where they create duplicates of or act on tasks from these 7. They are not mapped.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr"/>
-    </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>FINDINGS SUMMARY (live count from the Audit Findings sheet)</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="4">
+    <row r="33">
+      <c r="A33" s="4">
         <f>CONCATENATE("Confirmed: ",COUNTIF('Audit Findings'!B:B,"Confirmed"))</f>
         <v/>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="4">
+    <row r="34">
+      <c r="A34" s="4">
         <f>CONCATENATE("Potential Issue: ",COUNTIF('Audit Findings'!B:B,"Potential Issue"))</f>
         <v/>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="4">
+    <row r="35">
+      <c r="A35" s="4">
         <f>CONCATENATE("Needs Verification: ",COUNTIF('Audit Findings'!B:B,"Needs Verification"))</f>
         <v/>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="4">
+    <row r="36">
+      <c r="A36" s="4">
         <f>CONCATENATE("No Issue Found: ",COUNTIF('Audit Findings'!B:B,"No Issue Found"))</f>
         <v/>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>Sheets: Process Overview | Detailed Action Map | Workflow Inventory | Task &amp; Subtask Logic | Audit Findings | Evidence - Enrollments (one row per workflow run) | Evidence - Ticket Coverage (one row per ticket that entered a Transitions stage since 2026-08-20)</t>
         </is>
@@ -924,7 +931,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Enrollment trigger Needs Verification; observed match 21/21</t>
+          <t>VERIFIED (screenshot): Group 1 (all must be true): Create date is known AND Pipeline is any of Onboarding Pipeline AND Ticket status is any of Transition Kickoff (Onboarding Pipeline). No other groups (no OR).</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -934,7 +941,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Enrollment (INFERENCE: "ticket enters stage")</t>
+          <t>Enrollment: Records meet custom conditions (filter-based enrollment, not an event trigger)</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -2646,59 +2653,59 @@
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
+          <t>Group 1</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Enrollment trigger</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Records meet custom conditions (filter-based enrollment, not an event trigger)</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Enrolls a ticket when it meets: Group 1 (all must be true): Create date is known AND Pipeline is any of Onboarding Pipeline AND Ticket status is any of Transition Kickoff (Onboarding Pipeline). No other groups (no OR).</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Ticket</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>Create date; Pipeline; Ticket status (pipeline stage)</t>
+        </is>
+      </c>
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t>Pipeline = Onboarding Pipeline AND Ticket status = Transition Kickoff</t>
+        </is>
+      </c>
+      <c r="M4" s="6" t="inlineStr">
+        <is>
+          <t>The three conditions above, all required</t>
+        </is>
+      </c>
+      <c r="N4" s="6" t="inlineStr">
+        <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>Enrollment trigger</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>NEEDS VERIFICATION</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>NEEDS VERIFICATION. Observed: enrollment starts when the ticket enters "Transition Kickoff".</t>
-        </is>
-      </c>
-      <c r="I4" s="6" t="inlineStr">
-        <is>
-          <t>Ticket</t>
-        </is>
-      </c>
-      <c r="J4" s="6" t="inlineStr">
-        <is>
-          <t>Pipeline stage (hs_pipeline_stage)</t>
-        </is>
-      </c>
-      <c r="K4" s="6" t="inlineStr">
-        <is>
-          <t>Any earlier stage</t>
-        </is>
-      </c>
-      <c r="L4" s="6" t="inlineStr">
-        <is>
-          <t>Transition Kickoff (1094530721)</t>
-        </is>
-      </c>
-      <c r="M4" s="6" t="inlineStr">
-        <is>
-          <t>Needs Verification (re-enrollment and suppression unreadable)</t>
-        </is>
-      </c>
-      <c r="N4" s="6" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
       <c r="O4" s="6" t="inlineStr">
         <is>
           <t>21 enrollments on 21 tickets; no ticket enrolled twice.</t>
@@ -2711,17 +2718,17 @@
       </c>
       <c r="Q4" s="6" t="inlineStr">
         <is>
-          <t>21/21 enrollments started 4-13 seconds after the ticket's "Date entered Transition Kickoff" (hs_v2_date_entered_1094530721). Enrollments observed 2026-08-24 to 2026-10-01.</t>
+          <t>Screenshot of the enrollment trigger panel supplied by WLS on 2026-10-02. Matches the records: 21/21 enrollments started 4-13 seconds after the ticket's "Date entered Transition Kickoff" (hs_v2_date_entered_1094530721). Enrollments observed 2026-08-24 to 2026-10-01.</t>
         </is>
       </c>
       <c r="R4" s="6" t="inlineStr">
         <is>
-          <t>Ticket source does not matter: tickets created by the Closed Won workflow, by cloning and manually all enroll.</t>
-        </is>
-      </c>
-      <c r="S4" s="9" t="inlineStr">
-        <is>
-          <t>INFERENCE</t>
+          <t>Re-enrollment and suppression tabs not yet supplied - Needs Verification.</t>
+        </is>
+      </c>
+      <c r="S4" s="8" t="inlineStr">
+        <is>
+          <t>VERIFIED (screenshot)</t>
         </is>
       </c>
     </row>
@@ -6210,7 +6217,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>NEEDS VERIFICATION. Observed: ticket enters "Transition Kickoff" (stage ID 1094530721). 21/21 enrollments started 4-13 seconds after the ticket's "Date entered Transition Kickoff" (hs_v2_date_entered_1094530721). Enrollments observed 2026-08-24 to 2026-10-01.</t>
+          <t>VERIFIED (screenshot): Records meet custom conditions (filter-based enrollment, not an event trigger). Group 1 (all must be true): Create date is known AND Pipeline is any of Onboarding Pipeline AND Ticket status is any of Transition Kickoff (Onboarding Pipeline). No other groups (no OR).</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -14123,7 +14130,7 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Re-entering a stage re-creates the whole task set. Whether the (+SubTask) workflows also re-enroll is unknown - no ticket has re-entered a stage since they went live.</t>
+          <t>Re-entering a stage re-creates the whole task set. The (+SubTask) Kickoff trigger is filter-based (VERIFIED screenshot), so whether a ticket that re-enters Kickoff gets a second set depends on its re-enrollment setting, which has not been supplied. No ticket has re-entered a stage since the (+SubTask) workflows went live.</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
@@ -14217,12 +14224,12 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Shows that some condition (suppression, branch, or unenrollment) can stop the Kickoff workflow. That condition cannot be seen.</t>
+          <t>The trigger is filter-based (VERIFIED screenshot: Ticket status is any of Transition Kickoff). INFERENCE: the ticket left Kickoff 9 seconds after entering, before HubSpot evaluated it (other tickets enroll 4-13 s after entry), so it never met the conditions at evaluation time. Suppression is still unverified.</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>Check Kickoff suppression lists / "unenroll if criteria no longer met" and any Website Only exclusion.</t>
+          <t>Check Kickoff suppression lists. If the timing explanation is right, any ticket moved through Kickoff in under ~10 seconds will skip the Kickoff tasks.</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Record verified Kickoff workflow structure, re-enrollment and unenrollment settings
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TuFPqtNuPi7KBKeykeDCDb
</commit_message>
<xml_diff>
--- a/audits/transitions-workflow-audit/WLS_Transitions_Workflow_Audit.xlsx
+++ b/audits/transitions-workflow-audit/WLS_Transitions_Workflow_Audit.xlsx
@@ -2643,7 +2643,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Not exposed by HubSpot API - Needs Verification</t>
+          <t>1866384267</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -2698,7 +2698,7 @@
       </c>
       <c r="M4" s="6" t="inlineStr">
         <is>
-          <t>The three conditions above, all required</t>
+          <t>The three conditions above, all required. Re-enroll OFF; no unenroll criteria (VERIFIED)</t>
         </is>
       </c>
       <c r="N4" s="6" t="inlineStr">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="R4" s="6" t="inlineStr">
         <is>
-          <t>Re-enrollment and suppression tabs not yet supplied - Needs Verification.</t>
+          <t>Re-enrollment: OFF - "Allow tickets to re-enroll after completing the workflow" is switched off. Unenrollment/suppression: None - "Unenroll if tickets meet the following conditions" has no criteria (VERIFIED screenshot).</t>
         </is>
       </c>
       <c r="S4" s="8" t="inlineStr">
@@ -2740,17 +2740,17 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Not exposed by HubSpot API - Needs Verification</t>
+          <t>1866384267</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>1 (observed)</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Unknown (no branch evidence)</t>
+          <t>None (VERIFIED)</t>
         </is>
       </c>
       <c r="E5" s="6" t="n">
@@ -2758,17 +2758,17 @@
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>Create task, with subtasks (exact HubSpot label Needs Verification)</t>
+          <t>Create task</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>Task creation (observed output)</t>
+          <t>Create task (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>Creates parent task "Transition | TRANSITION KICK-OFF" with 14 subtask(s): 1. Respond to Customer Intro Email from Sales; 2. Review contract and setup internal handoff sales to PM for knowledge transfer; 3. Create customer folder in Google Drive; 4. Confirm Intake Form sent/completed; 5. Create Invoice for Setup Fee; 6. Schedule Onboarding Meeting with client (Client Meeting #1); 7. Complete Onboarding Meeting (and add link to populated Onboarding Form in HubSpot); 9. Submit BOG request in HubSpot to Hunter (if applicable, remote sites); 10. Submit Davinci lock order to Bryn in Hubspot (if required); 12. Send summary email to client; 13. Send email to collect client payment details (for Merchant Services and SafeLease); 15. Populate Playbook in Hubspot; 16. Confirm Setup Fee paid; 17. End of stage task sign off, Transition Kick Off.</t>
+          <t>Canvas reads: "Create task Transition | TRANSITION KICK-OFF with 14 subtasks and assign to Ticket owner" (VERIFIED). Records: parent "Transition | TRANSITION KICK-OFF" with 14 subtask(s): 1. Respond to Customer Intro Email from Sales; 2. Review contract and setup internal handoff sales to PM for knowledge transfer; 3. Create customer folder in Google Drive; 4. Confirm Intake Form sent/completed; 5. Create Invoice for Setup Fee; 6. Schedule Onboarding Meeting with client (Client Meeting #1); 7. Complete Onboarding Meeting (and add link to populated Onboarding Form in HubSpot); 9. Submit BOG request in HubSpot to Hunter (if applicable, remote sites); 10. Submit Davinci lock order to Bryn in Hubspot (if required); 12. Send summary email to client; 13. Send email to collect client payment details (for Merchant Services and SafeLease); 15. Populate Playbook in Hubspot; 16. Confirm Setup Fee paid; 17. End of stage task sign off, Transition Kick Off.</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
@@ -2788,17 +2788,17 @@
       </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
-          <t>Owner: Varies by ticket: Ryan Ashby (11/21); Hashem Haswah (10/21). Matches the ticket's current owner on 20/21 - consistent with "assign to ticket owner" (INFERENCE). Due: Most common: 7 business day(s) after creation date, at 08:00 US/Eastern (21/21 for days, 21/21 for time). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (20/21); Ticket (1/21).</t>
+          <t>Owner: Ticket owner (VERIFIED screenshot; records: Varies by ticket: Ryan Ashby (11/21); Hashem Haswah (10/21). Matches the ticket's current owner on 20/21 - consistent with "assign to ticket owner" (INFERENCE).) Due: Most common: 7 business day(s) after creation date, at 08:00 US/Eastern (21/21 for days, 21/21 for time). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (20/21); Ticket (1/21).</t>
         </is>
       </c>
       <c r="M5" s="6" t="inlineStr">
         <is>
-          <t>None observed - ran in every enrollment</t>
+          <t>None - no branches in this workflow (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="N5" s="6" t="inlineStr">
         <is>
-          <t>None observed: all tasks of one enrollment were created within 4 s.</t>
+          <t>None - no delay actions in this workflow (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="O5" s="6" t="inlineStr">
@@ -2823,7 +2823,7 @@
       </c>
       <c r="S5" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED (records) for output; action label NEEDS VERIFICATION</t>
+          <t>VERIFIED (screenshot + records); subtask owner/due/associations from records only</t>
         </is>
       </c>
     </row>
@@ -2835,17 +2835,17 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Not exposed by HubSpot API - Needs Verification</t>
+          <t>1866384267</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>2 (observed)</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Unknown (no branch evidence)</t>
+          <t>None (VERIFIED)</t>
         </is>
       </c>
       <c r="E6" s="6" t="n">
@@ -2853,17 +2853,17 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>Create task, with subtasks (exact HubSpot label Needs Verification)</t>
+          <t>Create task</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Task creation (observed output)</t>
+          <t>Create task (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>Creates parent task "Transition | TRANSITION KICK-OFF | Subtask - Mo'men" with 2 subtask(s): 8. Confirm GBP access OR Create a new GBP and grant relevant PoCs access (and initiate removal of duplicate with Google); 14. Check GBP verification, if GBP not verified: submit text verification and add email address (to GBP Profile) of individual who will be able to complete video verfication.</t>
+          <t>Canvas reads: "Create task Transition | TRANSITION KICK-OFF | Subtask - Mo'men with 2 subtasks and assign to Mo'men Khattab" (VERIFIED). Records: parent "Transition | TRANSITION KICK-OFF | Subtask - Mo'men" with 2 subtask(s): 8. Confirm GBP access OR Create a new GBP and grant relevant PoCs access (and initiate removal of duplicate with Google); 14. Check GBP verification, if GBP not verified: submit text verification and add email address (to GBP Profile) of individual who will be able to complete video verfication.</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
@@ -2883,17 +2883,17 @@
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>Owner: Mo'men Khattab on all 21 (looks like a fixed/static owner). Due: Most common: 7 business day(s) after creation date, at 08:00 US/Eastern (21/21 for days, 14/21 for time). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (20/21); Ticket (1/21).</t>
+          <t>Owner: Mo'men Khattab (VERIFIED screenshot; records: Mo'men Khattab on all 21 (looks like a fixed/static owner).) Due: Most common: 7 business day(s) after creation date, at 08:00 US/Eastern (21/21 for days, 14/21 for time). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (20/21); Ticket (1/21).</t>
         </is>
       </c>
       <c r="M6" s="6" t="inlineStr">
         <is>
-          <t>None observed - ran in every enrollment</t>
+          <t>None - no branches in this workflow (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="N6" s="6" t="inlineStr">
         <is>
-          <t>None observed: all tasks of one enrollment were created within 4 s.</t>
+          <t>None - no delay actions in this workflow (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="O6" s="6" t="inlineStr">
@@ -2914,7 +2914,7 @@
       <c r="R6" s="6" t="inlineStr"/>
       <c r="S6" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED (records) for output; action label NEEDS VERIFICATION</t>
+          <t>VERIFIED (screenshot + records); subtask owner/due/associations from records only</t>
         </is>
       </c>
     </row>
@@ -2926,17 +2926,17 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Not exposed by HubSpot API - Needs Verification</t>
+          <t>1866384267</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>3 (observed)</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Unknown (no branch evidence)</t>
+          <t>None (VERIFIED)</t>
         </is>
       </c>
       <c r="E7" s="6" t="n">
@@ -2944,17 +2944,17 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>Create task, with subtasks (exact HubSpot label Needs Verification)</t>
+          <t>Create task</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>Task creation (observed output)</t>
+          <t>Create task (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>Creates parent task "Transition | TRANSITION KICK-OFF | Subtask - Bryn" with 1 subtask(s): 11. Submit CSF/Toast form to Storable.</t>
+          <t>Canvas reads: "Create task Transition | TRANSITION KICK-OFF | Subtask - Bryn with 1 subtask and assign to Bryn Morgan" (VERIFIED). Records: parent "Transition | TRANSITION KICK-OFF | Subtask - Bryn" with 1 subtask(s): 11. Submit CSF/Toast form to Storable.</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
@@ -2974,17 +2974,17 @@
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>Owner: Bryn Morgan on all 21 (looks like a fixed/static owner). Due: Most common: 7 business day(s) after creation date, at 08:00 US/Eastern (9/21 for days, 9/21 for time). Other observed offsets: 11 bd x1, 14 bd x1, 15 bd x5, 19 bd x2, 20 bd x3 (could be manual due-date edits after creation - Needs Verification). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (21/21).</t>
+          <t>Owner: Bryn Morgan (VERIFIED screenshot; records: Bryn Morgan on all 21 (looks like a fixed/static owner).) Due: Most common: 7 business day(s) after creation date, at 08:00 US/Eastern (9/21 for days, 9/21 for time). Other observed offsets: 11 bd x1, 14 bd x1, 15 bd x5, 19 bd x2, 20 bd x3 (could be manual due-date edits after creation - Needs Verification). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (21/21).</t>
         </is>
       </c>
       <c r="M7" s="6" t="inlineStr">
         <is>
-          <t>None observed - ran in every enrollment</t>
+          <t>None - no branches in this workflow (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="N7" s="6" t="inlineStr">
         <is>
-          <t>None observed: all tasks of one enrollment were created within 4 s.</t>
+          <t>None - no delay actions in this workflow (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="O7" s="6" t="inlineStr">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="P7" s="6" t="inlineStr">
         <is>
-          <t>No further task-creating action observed. Anything after this (e.g. a property edit) is Needs Verification. Next process event: ticket moved to the next stage.</t>
+          <t>End (VERIFIED screenshot). Next process event: ticket moved to Pre-Launch Setup (manual - INFERENCE).</t>
         </is>
       </c>
       <c r="Q7" s="6" t="inlineStr">
@@ -3009,7 +3009,7 @@
       </c>
       <c r="S7" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED (records) for output; action label NEEDS VERIFICATION</t>
+          <t>VERIFIED (screenshot + records); subtask owner/due/associations from records only</t>
         </is>
       </c>
     </row>
@@ -6202,12 +6202,12 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Not exposed by HubSpot API - Needs Verification</t>
+          <t>1866384267 (ON, VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Ticket (INFERENCE: tasks are associated to the enrolled ticket)</t>
+          <t>Ticket (VERIFIED: "Trigger enrollment for tickets")</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
@@ -6222,17 +6222,17 @@
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>Needs Verification. Observed: 0 tickets enrolled more than once (so far no ticket has re-entered this stage after 2026-08-24).</t>
+          <t>VERIFIED (screenshot): OFF - "Allow tickets to re-enroll after completing the workflow" is switched off</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>Needs Verification. One possible effect seen in Kickoff: see Audit Findings F-07.</t>
+          <t>VERIFIED (screenshot): None - "Unenroll if tickets meet the following conditions" has no criteria</t>
         </is>
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>Needs Verification. At least 3 task-creating action(s) observed.</t>
+          <t>VERIFIED (screenshot): 3 actions, then End. No branches, no delays, no other action types</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr">
@@ -6717,12 +6717,12 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>Ticket enters Transition Kickoff (INFERENCE)</t>
+          <t>VERIFIED (screenshot): Group 1 (all must be true): Create date is known AND Pipeline is any of Onboarding Pipeline AND Ticket status is any of Transition Kickoff (Onboarding Pipeline). No other groups (no OR).</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>None observed - created in every enrollment</t>
+          <t>None - workflow has no branches (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="G2" s="6" t="inlineStr">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="N2" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED (records)</t>
+          <t>VERIFIED (screenshot: structure, parent owner) + records</t>
         </is>
       </c>
     </row>
@@ -6785,12 +6785,12 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Ticket enters Transition Kickoff (INFERENCE)</t>
+          <t>VERIFIED (screenshot): Group 1 (all must be true): Create date is known AND Pipeline is any of Onboarding Pipeline AND Ticket status is any of Transition Kickoff (Onboarding Pipeline). No other groups (no OR).</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>None observed - created in every enrollment</t>
+          <t>None - workflow has no branches (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr">
@@ -6828,7 +6828,7 @@
       </c>
       <c r="N3" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED (records)</t>
+          <t>VERIFIED (screenshot: structure, parent owner) + records</t>
         </is>
       </c>
     </row>
@@ -6853,12 +6853,12 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Ticket enters Transition Kickoff (INFERENCE)</t>
+          <t>VERIFIED (screenshot): Group 1 (all must be true): Create date is known AND Pipeline is any of Onboarding Pipeline AND Ticket status is any of Transition Kickoff (Onboarding Pipeline). No other groups (no OR).</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>None observed - created in every enrollment</t>
+          <t>None - workflow has no branches (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -6896,7 +6896,7 @@
       </c>
       <c r="N4" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED (records)</t>
+          <t>VERIFIED (screenshot: structure, parent owner) + records</t>
         </is>
       </c>
     </row>
@@ -6921,12 +6921,12 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Ticket enters Transition Kickoff (INFERENCE)</t>
+          <t>VERIFIED (screenshot): Group 1 (all must be true): Create date is known AND Pipeline is any of Onboarding Pipeline AND Ticket status is any of Transition Kickoff (Onboarding Pipeline). No other groups (no OR).</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>None observed - created in every enrollment</t>
+          <t>None - workflow has no branches (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="N5" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED (records)</t>
+          <t>VERIFIED (screenshot: structure, parent owner) + records</t>
         </is>
       </c>
     </row>
@@ -6989,12 +6989,12 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Ticket enters Transition Kickoff (INFERENCE)</t>
+          <t>VERIFIED (screenshot): Group 1 (all must be true): Create date is known AND Pipeline is any of Onboarding Pipeline AND Ticket status is any of Transition Kickoff (Onboarding Pipeline). No other groups (no OR).</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>None observed - created in every enrollment</t>
+          <t>None - workflow has no branches (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -7032,7 +7032,7 @@
       </c>
       <c r="N6" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED (records)</t>
+          <t>VERIFIED (screenshot: structure, parent owner) + records</t>
         </is>
       </c>
     </row>
@@ -7057,12 +7057,12 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Ticket enters Transition Kickoff (INFERENCE)</t>
+          <t>VERIFIED (screenshot): Group 1 (all must be true): Create date is known AND Pipeline is any of Onboarding Pipeline AND Ticket status is any of Transition Kickoff (Onboarding Pipeline). No other groups (no OR).</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>None observed - created in every enrollment</t>
+          <t>None - workflow has no branches (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -7100,7 +7100,7 @@
       </c>
       <c r="N7" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED (records)</t>
+          <t>VERIFIED (screenshot: structure, parent owner) + records</t>
         </is>
       </c>
     </row>
@@ -7125,12 +7125,12 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Ticket enters Transition Kickoff (INFERENCE)</t>
+          <t>VERIFIED (screenshot): Group 1 (all must be true): Create date is known AND Pipeline is any of Onboarding Pipeline AND Ticket status is any of Transition Kickoff (Onboarding Pipeline). No other groups (no OR).</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>None observed - created in every enrollment</t>
+          <t>None - workflow has no branches (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="N8" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED (records)</t>
+          <t>VERIFIED (screenshot: structure, parent owner) + records</t>
         </is>
       </c>
     </row>
@@ -7193,12 +7193,12 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Ticket enters Transition Kickoff (INFERENCE)</t>
+          <t>VERIFIED (screenshot): Group 1 (all must be true): Create date is known AND Pipeline is any of Onboarding Pipeline AND Ticket status is any of Transition Kickoff (Onboarding Pipeline). No other groups (no OR).</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>None observed - created in every enrollment</t>
+          <t>None - workflow has no branches (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
@@ -7236,7 +7236,7 @@
       </c>
       <c r="N9" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED (records)</t>
+          <t>VERIFIED (screenshot: structure, parent owner) + records</t>
         </is>
       </c>
     </row>
@@ -7261,12 +7261,12 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Ticket enters Transition Kickoff (INFERENCE)</t>
+          <t>VERIFIED (screenshot): Group 1 (all must be true): Create date is known AND Pipeline is any of Onboarding Pipeline AND Ticket status is any of Transition Kickoff (Onboarding Pipeline). No other groups (no OR).</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>None observed - created in every enrollment</t>
+          <t>None - workflow has no branches (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -7304,7 +7304,7 @@
       </c>
       <c r="N10" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED (records)</t>
+          <t>VERIFIED (screenshot: structure, parent owner) + records</t>
         </is>
       </c>
     </row>
@@ -7329,12 +7329,12 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Ticket enters Transition Kickoff (INFERENCE)</t>
+          <t>VERIFIED (screenshot): Group 1 (all must be true): Create date is known AND Pipeline is any of Onboarding Pipeline AND Ticket status is any of Transition Kickoff (Onboarding Pipeline). No other groups (no OR).</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>None observed - created in every enrollment</t>
+          <t>None - workflow has no branches (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="N11" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED (records)</t>
+          <t>VERIFIED (screenshot: structure, parent owner) + records</t>
         </is>
       </c>
     </row>
@@ -7397,12 +7397,12 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Ticket enters Transition Kickoff (INFERENCE)</t>
+          <t>VERIFIED (screenshot): Group 1 (all must be true): Create date is known AND Pipeline is any of Onboarding Pipeline AND Ticket status is any of Transition Kickoff (Onboarding Pipeline). No other groups (no OR).</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>None observed - created in every enrollment</t>
+          <t>None - workflow has no branches (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="N12" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED (records)</t>
+          <t>VERIFIED (screenshot: structure, parent owner) + records</t>
         </is>
       </c>
     </row>
@@ -7465,12 +7465,12 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Ticket enters Transition Kickoff (INFERENCE)</t>
+          <t>VERIFIED (screenshot): Group 1 (all must be true): Create date is known AND Pipeline is any of Onboarding Pipeline AND Ticket status is any of Transition Kickoff (Onboarding Pipeline). No other groups (no OR).</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>None observed - created in every enrollment</t>
+          <t>None - workflow has no branches (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
@@ -7508,7 +7508,7 @@
       </c>
       <c r="N13" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED (records)</t>
+          <t>VERIFIED (screenshot: structure, parent owner) + records</t>
         </is>
       </c>
     </row>
@@ -7533,12 +7533,12 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Ticket enters Transition Kickoff (INFERENCE)</t>
+          <t>VERIFIED (screenshot): Group 1 (all must be true): Create date is known AND Pipeline is any of Onboarding Pipeline AND Ticket status is any of Transition Kickoff (Onboarding Pipeline). No other groups (no OR).</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>None observed - created in every enrollment</t>
+          <t>None - workflow has no branches (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
@@ -7576,7 +7576,7 @@
       </c>
       <c r="N14" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED (records)</t>
+          <t>VERIFIED (screenshot: structure, parent owner) + records</t>
         </is>
       </c>
     </row>
@@ -7601,12 +7601,12 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Ticket enters Transition Kickoff (INFERENCE)</t>
+          <t>VERIFIED (screenshot): Group 1 (all must be true): Create date is known AND Pipeline is any of Onboarding Pipeline AND Ticket status is any of Transition Kickoff (Onboarding Pipeline). No other groups (no OR).</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>None observed - created in every enrollment</t>
+          <t>None - workflow has no branches (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
@@ -7644,7 +7644,7 @@
       </c>
       <c r="N15" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED (records)</t>
+          <t>VERIFIED (screenshot: structure, parent owner) + records</t>
         </is>
       </c>
     </row>
@@ -7669,12 +7669,12 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Ticket enters Transition Kickoff (INFERENCE)</t>
+          <t>VERIFIED (screenshot): Group 1 (all must be true): Create date is known AND Pipeline is any of Onboarding Pipeline AND Ticket status is any of Transition Kickoff (Onboarding Pipeline). No other groups (no OR).</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>None observed - created in every enrollment</t>
+          <t>None - workflow has no branches (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
@@ -7712,7 +7712,7 @@
       </c>
       <c r="N16" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED (records)</t>
+          <t>VERIFIED (screenshot: structure, parent owner) + records</t>
         </is>
       </c>
     </row>
@@ -7737,12 +7737,12 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Ticket enters Transition Kickoff (INFERENCE)</t>
+          <t>VERIFIED (screenshot): Group 1 (all must be true): Create date is known AND Pipeline is any of Onboarding Pipeline AND Ticket status is any of Transition Kickoff (Onboarding Pipeline). No other groups (no OR).</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>None observed - created in every enrollment</t>
+          <t>None - workflow has no branches (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="N17" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED (records)</t>
+          <t>VERIFIED (screenshot: structure, parent owner) + records</t>
         </is>
       </c>
     </row>
@@ -7805,12 +7805,12 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Ticket enters Transition Kickoff (INFERENCE)</t>
+          <t>VERIFIED (screenshot): Group 1 (all must be true): Create date is known AND Pipeline is any of Onboarding Pipeline AND Ticket status is any of Transition Kickoff (Onboarding Pipeline). No other groups (no OR).</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>None observed - created in every enrollment</t>
+          <t>None - workflow has no branches (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -7848,7 +7848,7 @@
       </c>
       <c r="N18" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED (records)</t>
+          <t>VERIFIED (screenshot: structure, parent owner) + records</t>
         </is>
       </c>
     </row>
@@ -7873,12 +7873,12 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Ticket enters Transition Kickoff (INFERENCE)</t>
+          <t>VERIFIED (screenshot): Group 1 (all must be true): Create date is known AND Pipeline is any of Onboarding Pipeline AND Ticket status is any of Transition Kickoff (Onboarding Pipeline). No other groups (no OR).</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>None observed - created in every enrollment</t>
+          <t>None - workflow has no branches (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
@@ -7916,7 +7916,7 @@
       </c>
       <c r="N19" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED (records)</t>
+          <t>VERIFIED (screenshot: structure, parent owner) + records</t>
         </is>
       </c>
     </row>
@@ -7941,12 +7941,12 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>Ticket enters Transition Kickoff (INFERENCE)</t>
+          <t>VERIFIED (screenshot): Group 1 (all must be true): Create date is known AND Pipeline is any of Onboarding Pipeline AND Ticket status is any of Transition Kickoff (Onboarding Pipeline). No other groups (no OR).</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>None observed - created in every enrollment</t>
+          <t>None - workflow has no branches (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
@@ -7984,7 +7984,7 @@
       </c>
       <c r="N20" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED (records)</t>
+          <t>VERIFIED (screenshot: structure, parent owner) + records</t>
         </is>
       </c>
     </row>
@@ -8009,12 +8009,12 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Ticket enters Transition Kickoff (INFERENCE)</t>
+          <t>VERIFIED (screenshot): Group 1 (all must be true): Create date is known AND Pipeline is any of Onboarding Pipeline AND Ticket status is any of Transition Kickoff (Onboarding Pipeline). No other groups (no OR).</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>None observed - created in every enrollment</t>
+          <t>None - workflow has no branches (VERIFIED screenshot)</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
@@ -8052,7 +8052,7 @@
       </c>
       <c r="N21" s="8" t="inlineStr">
         <is>
-          <t>VERIFIED (records)</t>
+          <t>VERIFIED (screenshot: structure, parent owner) + records</t>
         </is>
       </c>
     </row>
@@ -13932,7 +13932,7 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>HubSpot does not return the configuration of any of the 8 in-scope workflows through its API. Triggers, re-enrollment, suppression, branches, delays, non-task actions and action labels are all unverified.</t>
+          <t>HubSpot does not return the configuration of any of the 8 in-scope workflows through its API (Kickoff 1866384267 also returns 403). Kickoff is now verified from WLS screenshots (trigger, re-enrollment, unenrollment, canvas). For the other 7, triggers, re-enrollment, suppression, branches, delays, non-task actions and action labels remain unverified.</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
@@ -14130,12 +14130,12 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Re-entering a stage re-creates the whole task set. The (+SubTask) Kickoff trigger is filter-based (VERIFIED screenshot), so whether a ticket that re-enters Kickoff gets a second set depends on its re-enrollment setting, which has not been supplied. No ticket has re-entered a stage since the (+SubTask) workflows went live.</t>
+          <t>The legacy workflow re-created the whole task set on re-entry. The (+SubTask) Kickoff workflow has Re-enroll OFF (VERIFIED screenshot), so it will NOT create duplicates - but a ticket that returns to Transition Kickoff (e.g. after On Hold) will get NO new Kickoff tasks. Its original tasks (possibly completed or old) are all it has.</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>Check the re-enrollment setting on all 7 (+SubTask) workflows.</t>
+          <t>Decide whether a ticket returning to Kickoff should get fresh tasks. Check the re-enrollment setting on the other 6 (+SubTask) workflows.</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
@@ -14197,9 +14197,9 @@
           <t>F-07</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Needs Verification</t>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Potential Issue</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -14224,12 +14224,12 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>The trigger is filter-based (VERIFIED screenshot: Ticket status is any of Transition Kickoff). INFERENCE: the ticket left Kickoff 9 seconds after entering, before HubSpot evaluated it (other tickets enroll 4-13 s after entry), so it never met the conditions at evaluation time. Suppression is still unverified.</t>
+          <t>Suppression and unenrollment are ruled out: Kickoff has no unenroll criteria and no branches (VERIFIED screenshot). The trigger is filter-based (Ticket status is any of Transition Kickoff). INFERENCE: the ticket left Kickoff 9 seconds after entering, before HubSpot evaluated it (other tickets enroll 4-13 s after entry), so it never met the conditions at evaluation time.</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>Check Kickoff suppression lists. If the timing explanation is right, any ticket moved through Kickoff in under ~10 seconds will skip the Kickoff tasks.</t>
+          <t>Check the ticket's workflow history (Kickoff &gt; Performance history) to confirm it was never enrolled. Any ticket moved through Kickoff in under ~10 seconds will skip the Kickoff tasks.</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
@@ -14553,7 +14553,7 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Named owners are probably hard-coded (INFERENCE). If someone leaves or changes role, new tasks still go to them.</t>
+          <t>Named owners are probably hard-coded (INFERENCE). Kickoff confirms it: Action 1 "assign to Ticket owner", Action 2 "assign to Mo'men Khattab", Action 3 "assign to Bryn Morgan" (VERIFIED screenshot). If someone leaves or changes role, new tasks still go to them.</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Record verified Kickoff Action 1 settings and association findings
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TuFPqtNuPi7KBKeykeDCDb
</commit_message>
<xml_diff>
--- a/audits/transitions-workflow-audit/WLS_Transitions_Workflow_Audit.xlsx
+++ b/audits/transitions-workflow-audit/WLS_Transitions_Workflow_Audit.xlsx
@@ -21,7 +21,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Detailed Action Map'!$A$1:$S$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Workflow Inventory'!$A$1:$K$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Task &amp; Subtask Logic'!$A$1:$N$106</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Audit Findings'!$A$1:$I$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Audit Findings'!$A$1:$I$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Evidence - Enrollments'!$A$1:$N$102</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Evidence - Ticket Coverage'!$A$1:$M$67</definedName>
   </definedNames>
@@ -2788,7 +2788,7 @@
       </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
-          <t>Owner: Ticket owner (VERIFIED screenshot; records: Varies by ticket: Ryan Ashby (11/21); Hashem Haswah (10/21). Matches the ticket's current owner on 20/21 - consistent with "assign to ticket owner" (INFERENCE).) Due: Most common: 7 business day(s) after creation date, at 08:00 US/Eastern (21/21 for days, 21/21 for time). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (20/21); Ticket (1/21).</t>
+          <t>VERIFIED CONFIG: Title "Transition | TRANSITION KICK-OFF"; Type To-do; Start date Immediately; Due date Custom: 7 days at 8:00 AM, Business days only (Mon-Fri), account time zone UTC-04:00; Email reminder None; Shared task queue None; Priority (None); Assign task to "An existing owner of the ticket" -&gt; Ticket owner; Notes: "Before You Begin: Stage entered - Master Task created (TRANSITION KICK-OFF); Waiting for Customer - Customer must pay the Setup Fee invoiced in item 5; Waiting for Other - All Kick-Off subtasks (PM, Momen, Bryn) must be complete. Before Completing This Task: Verify all checklist items are complete; Notify PM if blockers exist; Mark task Complete"; Subtasks (14, titles only shown in panel): 1, 2, 3, 4, 5, 6, 7, 9, 10, 12, 13, 15, 16, 17; Associate new task with: the enrolled ticket + associated contacts with label "Transition" + All associated companies. RECORDS: Owner: Ticket owner (VERIFIED screenshot; records: Varies by ticket: Ryan Ashby (11/21); Hashem Haswah (10/21). Matches the ticket's current owner on 20/21 - consistent with "assign to ticket owner" (INFERENCE).) Due: Most common: 7 business day(s) after creation date, at 08:00 US/Eastern (21/21 for days, 21/21 for time). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (20/21); Ticket (1/21).</t>
         </is>
       </c>
       <c r="M5" s="6" t="inlineStr">
@@ -6727,7 +6727,7 @@
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>Owner: Varies by ticket: Ryan Ashby (11/21); Hashem Haswah (10/21). Matches the ticket's current owner on 20/21 - consistent with "assign to ticket owner" (INFERENCE). Due: Most common: 7 business day(s) after creation date, at 08:00 US/Eastern (21/21 for days, 21/21 for time). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (20/21); Ticket (1/21).</t>
+          <t>VERIFIED CONFIG (Screenshots of the Action 1 edit panel supplied by WLS on 2026-10-02): Title "Transition | TRANSITION KICK-OFF"; Type To-do; Start date Immediately; Due date Custom: 7 days at 8:00 AM, Business days only (Mon-Fri), account time zone UTC-04:00; Email reminder None; Shared task queue None; Priority (None); Assign task to "An existing owner of the ticket" -&gt; Ticket owner; Notes: "Before You Begin: Stage entered - Master Task created (TRANSITION KICK-OFF); Waiting for Customer - Customer must pay the Setup Fee invoiced in item 5; Waiting for Other - All Kick-Off subtasks (PM, Momen, Bryn) must be complete. Before Completing This Task: Verify all checklist items are complete; Notify PM if blockers exist; Mark task Complete"; Subtasks (14, titles only shown in panel): 1, 2, 3, 4, 5, 6, 7, 9, 10, 12, 13, 15, 16, 17; Associate new task with: the enrolled ticket + associated contacts with label "Transition" + All associated companies. RECORDS: Owner: Varies by ticket: Ryan Ashby (11/21); Hashem Haswah (10/21). Matches the ticket's current owner on 20/21 - consistent with "assign to ticket owner" (INFERENCE). Due: Most common: 7 business day(s) after creation date, at 08:00 US/Eastern (21/21 for days, 21/21 for time). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (20/21); Ticket (1/21).</t>
         </is>
       </c>
       <c r="H2" s="6" t="inlineStr">
@@ -6737,7 +6737,7 @@
       </c>
       <c r="I2" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Task notes (VERIFIED) say: wait for the customer to pay the Setup Fee (subtask 5) and for all Kick-Off subtasks incl. Mo'men's and Bryn's parents to be complete. This is an instruction only - nothing in the workflow enforces it.</t>
         </is>
       </c>
       <c r="J2" s="6" t="inlineStr">
@@ -6800,7 +6800,7 @@
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>Owner: No owner on any of the 21 subtasks. Due: Most common: 1 business day(s) after creation date, at 08:00 US/Eastern (18/21 for days, 21/21 for time). Other observed offsets: 3 bd x3 (could be manual due-date edits after creation - Needs Verification). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (16/21); Ticket (5/21).</t>
+          <t>Title VERIFIED in action config (subtask owner/due settings not shown in the panel - Needs Verification). RECORDS: Owner: No owner on any of the 21 subtasks. Due: Most common: 1 business day(s) after creation date, at 08:00 US/Eastern (18/21 for days, 21/21 for time). Other observed offsets: 3 bd x3 (could be manual due-date edits after creation - Needs Verification). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (16/21); Ticket (5/21).</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr">
@@ -6868,7 +6868,7 @@
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>Owner: No owner on any of the 21 subtasks. Due: Most common: 2 business day(s) after creation date, at 08:00 US/Eastern (18/21 for days, 21/21 for time). Other observed offsets: 3 bd x3 (could be manual due-date edits after creation - Needs Verification). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (16/21); Ticket (5/21).</t>
+          <t>Title VERIFIED in action config (subtask owner/due settings not shown in the panel - Needs Verification). RECORDS: Owner: No owner on any of the 21 subtasks. Due: Most common: 2 business day(s) after creation date, at 08:00 US/Eastern (18/21 for days, 21/21 for time). Other observed offsets: 3 bd x3 (could be manual due-date edits after creation - Needs Verification). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (16/21); Ticket (5/21).</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
@@ -6936,7 +6936,7 @@
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>Owner: No owner on any of the 21 subtasks. Due: Most common: 2 business day(s) after creation date, at 08:00 US/Eastern (17/21 for days, 21/21 for time). Other observed offsets: 3 bd x3, 6 bd x1 (could be manual due-date edits after creation - Needs Verification). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (16/21); Ticket (5/21).</t>
+          <t>Title VERIFIED in action config (subtask owner/due settings not shown in the panel - Needs Verification). RECORDS: Owner: No owner on any of the 21 subtasks. Due: Most common: 2 business day(s) after creation date, at 08:00 US/Eastern (17/21 for days, 21/21 for time). Other observed offsets: 3 bd x3, 6 bd x1 (could be manual due-date edits after creation - Needs Verification). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (16/21); Ticket (5/21).</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
@@ -7004,7 +7004,7 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>Owner: No owner on any of the 21 subtasks. Due: Most common: 2 business day(s) after creation date, at 08:00 US/Eastern (17/21 for days, 21/21 for time). Other observed offsets: 3 bd x3, 6 bd x1 (could be manual due-date edits after creation - Needs Verification). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (16/21); Ticket (5/21).</t>
+          <t>Title VERIFIED in action config (subtask owner/due settings not shown in the panel - Needs Verification). RECORDS: Owner: No owner on any of the 21 subtasks. Due: Most common: 2 business day(s) after creation date, at 08:00 US/Eastern (17/21 for days, 21/21 for time). Other observed offsets: 3 bd x3, 6 bd x1 (could be manual due-date edits after creation - Needs Verification). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (16/21); Ticket (5/21).</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
@@ -7072,7 +7072,7 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>Owner: No owner on any of the 21 subtasks. Due: Most common: 2 business day(s) after creation date, at 08:00 US/Eastern (18/21 for days, 21/21 for time). Other observed offsets: 3 bd x3 (could be manual due-date edits after creation - Needs Verification). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (16/21); Ticket (5/21).</t>
+          <t>Title VERIFIED in action config (subtask owner/due settings not shown in the panel - Needs Verification). RECORDS: Owner: No owner on any of the 21 subtasks. Due: Most common: 2 business day(s) after creation date, at 08:00 US/Eastern (18/21 for days, 21/21 for time). Other observed offsets: 3 bd x3 (could be manual due-date edits after creation - Needs Verification). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (16/21); Ticket (5/21).</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
@@ -7140,7 +7140,7 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>Owner: No owner on any of the 21 subtasks. Due: Most common: 3 business day(s) after creation date, at 08:00 US/Eastern (20/21 for days, 21/21 for time). Other observed offsets: 6 bd x1 (could be manual due-date edits after creation - Needs Verification). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (16/21); Ticket (5/21).</t>
+          <t>Title VERIFIED in action config (subtask owner/due settings not shown in the panel - Needs Verification). RECORDS: Owner: No owner on any of the 21 subtasks. Due: Most common: 3 business day(s) after creation date, at 08:00 US/Eastern (20/21 for days, 21/21 for time). Other observed offsets: 6 bd x1 (could be manual due-date edits after creation - Needs Verification). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (16/21); Ticket (5/21).</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
@@ -7208,7 +7208,7 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>Owner: No owner on any of the 21 subtasks. Due: Most common: 5 business day(s) after creation date, at 08:00 US/Eastern (21/21 for days, 21/21 for time). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (16/21); Ticket (5/21).</t>
+          <t>Title VERIFIED in action config (subtask owner/due settings not shown in the panel - Needs Verification). RECORDS: Owner: No owner on any of the 21 subtasks. Due: Most common: 5 business day(s) after creation date, at 08:00 US/Eastern (21/21 for days, 21/21 for time). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (16/21); Ticket (5/21).</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
@@ -7276,7 +7276,7 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>Owner: No owner on any of the 21 subtasks. Due: Most common: 6 business day(s) after creation date, at 08:00 US/Eastern (21/21 for days, 21/21 for time). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (16/21); Ticket (5/21).</t>
+          <t>Title VERIFIED in action config (subtask owner/due settings not shown in the panel - Needs Verification). RECORDS: Owner: No owner on any of the 21 subtasks. Due: Most common: 6 business day(s) after creation date, at 08:00 US/Eastern (21/21 for days, 21/21 for time). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (16/21); Ticket (5/21).</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
@@ -7344,7 +7344,7 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>Owner: No owner on any of the 21 subtasks. Due: Most common: 6 business day(s) after creation date, at 08:00 US/Eastern (21/21 for days, 21/21 for time). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (16/21); Ticket (5/21).</t>
+          <t>Title VERIFIED in action config (subtask owner/due settings not shown in the panel - Needs Verification). RECORDS: Owner: No owner on any of the 21 subtasks. Due: Most common: 6 business day(s) after creation date, at 08:00 US/Eastern (21/21 for days, 21/21 for time). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (16/21); Ticket (5/21).</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
@@ -7412,7 +7412,7 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>Owner: No owner on any of the 21 subtasks. Due: Most common: 6 business day(s) after creation date, at 08:00 US/Eastern (21/21 for days, 21/21 for time). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (16/21); Ticket (5/21).</t>
+          <t>Title VERIFIED in action config (subtask owner/due settings not shown in the panel - Needs Verification). RECORDS: Owner: No owner on any of the 21 subtasks. Due: Most common: 6 business day(s) after creation date, at 08:00 US/Eastern (21/21 for days, 21/21 for time). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (16/21); Ticket (5/21).</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
@@ -7480,7 +7480,7 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>Owner: No owner on any of the 21 subtasks. Due: Most common: 6 business day(s) after creation date, at 08:00 US/Eastern (21/21 for days, 21/21 for time). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (16/21); Ticket (5/21).</t>
+          <t>Title VERIFIED in action config (subtask owner/due settings not shown in the panel - Needs Verification). RECORDS: Owner: No owner on any of the 21 subtasks. Due: Most common: 6 business day(s) after creation date, at 08:00 US/Eastern (21/21 for days, 21/21 for time). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (16/21); Ticket (5/21).</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
@@ -7548,7 +7548,7 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>Owner: No owner on any of the 21 subtasks. Due: Most common: 7 business day(s) after creation date, at 08:00 US/Eastern (21/21 for days, 21/21 for time). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (16/21); Ticket (5/21).</t>
+          <t>Title VERIFIED in action config (subtask owner/due settings not shown in the panel - Needs Verification). RECORDS: Owner: No owner on any of the 21 subtasks. Due: Most common: 7 business day(s) after creation date, at 08:00 US/Eastern (21/21 for days, 21/21 for time). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (16/21); Ticket (5/21).</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
@@ -7616,7 +7616,7 @@
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>Owner: No owner on any of the 21 subtasks. Due: Most common: 7 business day(s) after creation date, at 08:00 US/Eastern (21/21 for days, 21/21 for time). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (16/21); Ticket (5/21).</t>
+          <t>Title VERIFIED in action config (subtask owner/due settings not shown in the panel - Needs Verification). RECORDS: Owner: No owner on any of the 21 subtasks. Due: Most common: 7 business day(s) after creation date, at 08:00 US/Eastern (21/21 for days, 21/21 for time). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (16/21); Ticket (5/21).</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
@@ -7684,7 +7684,7 @@
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>Owner: No owner on any of the 21 subtasks. Due: Most common: 7 business day(s) after creation date, at 08:00 US/Eastern (21/21 for days, 21/21 for time). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (19/21); Ticket (2/21).</t>
+          <t>Title VERIFIED in action config (subtask owner/due settings not shown in the panel - Needs Verification). RECORDS: Owner: No owner on any of the 21 subtasks. Due: Most common: 7 business day(s) after creation date, at 08:00 US/Eastern (21/21 for days, 21/21 for time). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (19/21); Ticket (2/21).</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
@@ -7747,7 +7747,7 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Owner: Mo'men Khattab on all 21 (looks like a fixed/static owner). Due: Most common: 7 business day(s) after creation date, at 08:00 US/Eastern (21/21 for days, 14/21 for time). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (20/21); Ticket (1/21).</t>
+          <t>VERIFIED (canvas): assigned to Mo'men Khattab. RECORDS: Owner: Mo'men Khattab on all 21 (looks like a fixed/static owner). Due: Most common: 7 business day(s) after creation date, at 08:00 US/Eastern (21/21 for days, 14/21 for time). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (20/21); Ticket (1/21).</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
@@ -7951,7 +7951,7 @@
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Owner: Bryn Morgan on all 21 (looks like a fixed/static owner). Due: Most common: 7 business day(s) after creation date, at 08:00 US/Eastern (9/21 for days, 9/21 for time). Other observed offsets: 11 bd x1, 14 bd x1, 15 bd x5, 19 bd x2, 20 bd x3 (could be manual due-date edits after creation - Needs Verification). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (21/21).</t>
+          <t>VERIFIED (canvas): assigned to Bryn Morgan. RECORDS: Owner: Bryn Morgan on all 21 (looks like a fixed/static owner). Due: Most common: 7 business day(s) after creation date, at 08:00 US/Eastern (9/21 for days, 9/21 for time). Other observed offsets: 11 bd x1, 14 bd x1, 15 bd x5, 19 bd x2, 20 bd x3 (could be manual due-date edits after creation - Needs Verification). Priority: NONE (21/21). Type: TODO (21/21). Associations: Ticket + Company (21/21).</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
@@ -13848,7 +13848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -14996,39 +14996,39 @@
           <t>F-24</t>
         </is>
       </c>
-      <c r="B25" s="10" t="inlineStr">
-        <is>
-          <t>No Issue Found</t>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>All 7 (+SubTask)</t>
+          <t>Transitions - Transition Kickoff Tasks (+SubTask)</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Enrollment</t>
+          <t>Action #1 associations</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Every ticket whose latest entry into a stage is after the matching (+SubTask) workflow went live got exactly one enrollment, with the single exception in F-07 (based on the latest "Date entered" value per stage; earlier entries are overwritten). No delays between task actions (all tasks of an enrollment created within ~1-85 seconds).</t>
+          <t>The contact association never adds anyone. Action 1 is set to associate "associated contacts" with label "Transition" (VERIFIED screenshot), but none of the 420 Kickoff tasks is linked to a contact. All 21 Kickoff tickets do have contacts, but none of those ticket-contact associations carries the "Transition" label (they are all unlabelled).</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>Enrollment evidence sheet; stage-entry dates of all 262 Onboarding Pipeline tickets.</t>
+          <t>Action 1 panel: "Associated contacts - Associate Transition". Ticket-&gt;contact association labels on the 21 Kickoff tickets: 21 unlabelled, 0 "Transition" (label typeId 72 exists). Task-&gt;contact associations: 0/420.</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>Task creation itself is reliable once a ticket reaches a stage.</t>
+          <t>Kickoff tasks never appear on the customer contact's record, although the setting suggests they should.</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>Decide whether to label the main customer contact "Transition" on each ticket, or change the action to all associated contacts.</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
@@ -15043,39 +15043,39 @@
           <t>F-25</t>
         </is>
       </c>
-      <c r="B26" s="8" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Needs Verification</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Set task queue (1677143128) + Kickoff (+SubTask) + Launch Readiness (+SubTask)</t>
+          <t>Transitions - Transition Kickoff Tasks (+SubTask)</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>Kickoff #1 subtask 9; Launch Readiness #2 subtask 2</t>
+          <t>Action #1 subtasks</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>A different workflow moves two Transitions subtasks into the "BOG - Run and Sustain" task queue. "Set task queue" (readable, ON) enrolls every newly created task and, if the title contains "BOG", sets Queue = 9999918 (its "BOG - Run and Sustain" branch). "9. Submit BOG request in HubSpot to Hunter" (21/21) and "2. Finalize BOG candidates, paperwork, details in Hubspot" (20/20) are in that queue; no other Transitions task is in any queue.</t>
+          <t>Action 1 is set to associate the task with all associated companies (VERIFIED screenshot). The parent got the company in 20/21 enrollments, but in the 4 earliest enrollments (2026-08-24 to 08-27) 13-14 of its 14 subtasks got no company, while the parent did. From 2026-08-28 subtasks get the company too. (The 2026-09-01 ticket had no company at all.)</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>Config of workflow 1677143128 (VERIFIED: list branch "BOG - Run and Sustain" -&gt; action 3 sets hs_queue_membership_ids = 9999918). Task records: hs_queue_membership_ids = 9999918 on exactly those 41 subtasks.</t>
+          <t>Task-&gt;company associations of Kickoff Action #1 subtasks vs. their parent, by enrollment date.</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>Onboarding subtasks with no owner show up in a Run &amp; Sustain queue. That may be how Hunter's team finds them, or it may be unintended.</t>
+          <t>Suggests subtasks did not inherit the parent's associations until about 2026-08-28 (a HubSpot or workflow change). Older subtasks do not show on the company record.</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>Confirm with the BOG team whether onboarding subtasks should be in the Run &amp; Sustain queue.</t>
+          <t>No action needed if the current behaviour is right; optionally add the company to the ~70 older subtasks.</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
@@ -15090,49 +15090,190 @@
           <t>F-26</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Needs Verification</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Transitions - Transition Kickoff Tasks (+SubTask)</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>Action #1 subtasks</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>Subtask due dates: the parent is due in 7 business days at 8:00 AM (VERIFIED, matches 21/21 records), but its subtasks are due 1-7 business days after creation (e.g. subtask 1 in 1 bd, subtask 7 in 5 bd, subtask 17 in 7 bd). The action panel lists only the subtask titles, so where these per-subtask due dates and the "no owner" setting come from is not visible.</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>Action 1 panel (Due date 7, business days only); subtask due dates in records (Task &amp; Subtask Logic).</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>Needed to confirm F-02 (subtasks without owners) is a setting, not a side effect.</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>Click one subtask inside Action 1 and screenshot its settings (owner and due date).</t>
+        </is>
+      </c>
+      <c r="I27" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>F-27</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>No Issue Found</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>All 7 (+SubTask)</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>Enrollment</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>Every ticket whose latest entry into a stage is after the matching (+SubTask) workflow went live got exactly one enrollment, with the single exception in F-07 (based on the latest "Date entered" value per stage; earlier entries are overwritten). No delays between task actions (all tasks of an enrollment created within ~1-85 seconds).</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>Enrollment evidence sheet; stage-entry dates of all 262 Onboarding Pipeline tickets.</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>Task creation itself is reliable once a ticket reaches a stage.</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>F-28</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Set task queue (1677143128) + Kickoff (+SubTask) + Launch Readiness (+SubTask)</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>Kickoff #1 subtask 9; Launch Readiness #2 subtask 2</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>A different workflow moves two Transitions subtasks into the "BOG - Run and Sustain" task queue. "Set task queue" (readable, ON) enrolls every newly created task and, if the title contains "BOG", sets Queue = 9999918 (its "BOG - Run and Sustain" branch). "9. Submit BOG request in HubSpot to Hunter" (21/21) and "2. Finalize BOG candidates, paperwork, details in Hubspot" (20/20) are in that queue; no other Transitions task is in any queue.</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>Config of workflow 1677143128 (VERIFIED: list branch "BOG - Run and Sustain" -&gt; action 3 sets hs_queue_membership_ids = 9999918). Task records: hs_queue_membership_ids = 9999918 on exactly those 41 subtasks.</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>Onboarding subtasks with no owner show up in a Run &amp; Sustain queue. That may be how Hunter's team finds them, or it may be unintended.</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>Confirm with the BOG team whether onboarding subtasks should be in the Run &amp; Sustain queue.</t>
+        </is>
+      </c>
+      <c r="I29" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>F-29</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>Potential Issue</t>
         </is>
       </c>
-      <c r="C27" s="6" t="inlineStr">
+      <c r="C30" s="6" t="inlineStr">
         <is>
           <t>Set OM and SM overdue tasks to Deferred (1795953061) + all 7 (+SubTask)</t>
         </is>
       </c>
-      <c r="D27" s="6" t="inlineStr">
+      <c r="D30" s="6" t="inlineStr">
         <is>
           <t>Parent tasks owned by OM/SM team members</t>
         </is>
       </c>
-      <c r="E27" s="6" t="inlineStr">
+      <c r="E30" s="6" t="inlineStr">
         <is>
           <t>A different workflow can defer Transitions tasks automatically. "Set OM and SM overdue tasks to Deferred" (readable, ON) sets Status = DEFERRED on overdue, not-completed tasks whose owner team is 58458611 or 58458777. The 4 DEFERRED Transitions tasks are all "Transition | LAUNCH READINESS | Subtask - Hunter" parents (owner Hunter Stoner) (INFERENCE: deferred by this workflow; the team names/members could not be read - scope settings.users.teams.read missing). Subtasks have no owner, so this workflow can never act on them.</t>
         </is>
       </c>
-      <c r="F27" s="6" t="inlineStr">
+      <c r="F30" s="6" t="inlineStr">
         <is>
           <t>Config of workflow 1795953061 (VERIFIED: enrollment = hs_task_is_overdue true AND hubspot_team_id in [58458611, 58458777] AND status not Completed; action 1 sets hs_task_status = DEFERRED). Task records: 4 DEFERRED parents, all owner 80038421.</t>
         </is>
       </c>
-      <c r="G27" s="6" t="inlineStr">
+      <c r="G30" s="6" t="inlineStr">
         <is>
           <t>A deferred Launch Readiness parent drops out of overdue views while its subtask (2. Finalize BOG candidates) can still be open.</t>
         </is>
       </c>
-      <c r="H27" s="6" t="inlineStr">
+      <c r="H30" s="6" t="inlineStr">
         <is>
           <t>Confirm which users are in teams 58458611 / 58458777 and whether Transitions tasks should be excluded from auto-deferral.</t>
         </is>
       </c>
-      <c r="I27" s="6" t="inlineStr">
+      <c r="I30" s="6" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I27"/>
+  <autoFilter ref="A1:I30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Keep finding numbers stable; fix cross-references
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TuFPqtNuPi7KBKeykeDCDb
</commit_message>
<xml_diff>
--- a/audits/transitions-workflow-audit/WLS_Transitions_Workflow_Audit.xlsx
+++ b/audits/transitions-workflow-audit/WLS_Transitions_Workflow_Audit.xlsx
@@ -2818,7 +2818,7 @@
       </c>
       <c r="R5" s="6" t="inlineStr">
         <is>
-          <t>WORKFLOW HANDOFF: "Set task queue" (1677143128) then puts subtask "9. Submit BOG request in HubSpot to Hunter (if applicable, remote sites)" into queue "BOG - Run and Sustain" (VERIFIED config + records, see F-24).</t>
+          <t>WORKFLOW HANDOFF: "Set task queue" (1677143128) then puts subtask "9. Submit BOG request in HubSpot to Hunter (if applicable, remote sites)" into queue "BOG - Run and Sustain" (VERIFIED config + records, see F-25).</t>
         </is>
       </c>
       <c r="S5" s="8" t="inlineStr">
@@ -4104,7 +4104,7 @@
       </c>
       <c r="R19" s="6" t="inlineStr">
         <is>
-          <t>WORKFLOW HANDOFF: "Set task queue" (1677143128) then puts subtask "2. Finalize BOG candidates, paperwork, details in Hubspot" into queue "BOG - Run and Sustain" (VERIFIED config + records, see F-24). WORKFLOW HANDOFF: "Set OM and SM overdue tasks to Deferred" (1795953061) can set this parent to DEFERRED once overdue (4 observed, see F-25).</t>
+          <t>WORKFLOW HANDOFF: "Set task queue" (1677143128) then puts subtask "2. Finalize BOG candidates, paperwork, details in Hubspot" into queue "BOG - Run and Sustain" (VERIFIED config + records, see F-25). WORKFLOW HANDOFF: "Set OM and SM overdue tasks to Deferred" (1795953061) can set this parent to DEFERRED once overdue (4 observed, see F-26).</t>
         </is>
       </c>
       <c r="S19" s="8" t="inlineStr">
@@ -14996,39 +14996,39 @@
           <t>F-24</t>
         </is>
       </c>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>No Issue Found</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Transitions - Transition Kickoff Tasks (+SubTask)</t>
+          <t>All 7 (+SubTask)</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Action #1 associations</t>
+          <t>Enrollment</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>The contact association never adds anyone. Action 1 is set to associate "associated contacts" with label "Transition" (VERIFIED screenshot), but none of the 420 Kickoff tasks is linked to a contact. All 21 Kickoff tickets do have contacts, but none of those ticket-contact associations carries the "Transition" label (they are all unlabelled).</t>
+          <t>Every ticket whose latest entry into a stage is after the matching (+SubTask) workflow went live got exactly one enrollment, with the single exception in F-07 (based on the latest "Date entered" value per stage; earlier entries are overwritten). No delays between task actions (all tasks of an enrollment created within ~1-85 seconds).</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>Action 1 panel: "Associated contacts - Associate Transition". Ticket-&gt;contact association labels on the 21 Kickoff tickets: 21 unlabelled, 0 "Transition" (label typeId 72 exists). Task-&gt;contact associations: 0/420.</t>
+          <t>Enrollment evidence sheet; stage-entry dates of all 262 Onboarding Pipeline tickets.</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>Kickoff tasks never appear on the customer contact's record, although the setting suggests they should.</t>
+          <t>Task creation itself is reliable once a ticket reaches a stage.</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>Decide whether to label the main customer contact "Transition" on each ticket, or change the action to all associated contacts.</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
@@ -15043,39 +15043,39 @@
           <t>F-25</t>
         </is>
       </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>Needs Verification</t>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Transitions - Transition Kickoff Tasks (+SubTask)</t>
+          <t>Set task queue (1677143128) + Kickoff (+SubTask) + Launch Readiness (+SubTask)</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>Action #1 subtasks</t>
+          <t>Kickoff #1 subtask 9; Launch Readiness #2 subtask 2</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>Action 1 is set to associate the task with all associated companies (VERIFIED screenshot). The parent got the company in 20/21 enrollments, but in the 4 earliest enrollments (2026-08-24 to 08-27) 13-14 of its 14 subtasks got no company, while the parent did. From 2026-08-28 subtasks get the company too. (The 2026-09-01 ticket had no company at all.)</t>
+          <t>A different workflow moves two Transitions subtasks into the "BOG - Run and Sustain" task queue. "Set task queue" (readable, ON) enrolls every newly created task and, if the title contains "BOG", sets Queue = 9999918 (its "BOG - Run and Sustain" branch). "9. Submit BOG request in HubSpot to Hunter" (21/21) and "2. Finalize BOG candidates, paperwork, details in Hubspot" (20/20) are in that queue; no other Transitions task is in any queue.</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>Task-&gt;company associations of Kickoff Action #1 subtasks vs. their parent, by enrollment date.</t>
+          <t>Config of workflow 1677143128 (VERIFIED: list branch "BOG - Run and Sustain" -&gt; action 3 sets hs_queue_membership_ids = 9999918). Task records: hs_queue_membership_ids = 9999918 on exactly those 41 subtasks.</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>Suggests subtasks did not inherit the parent's associations until about 2026-08-28 (a HubSpot or workflow change). Older subtasks do not show on the company record.</t>
+          <t>Onboarding subtasks with no owner show up in a Run &amp; Sustain queue. That may be how Hunter's team finds them, or it may be unintended.</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>No action needed if the current behaviour is right; optionally add the company to the ~70 older subtasks.</t>
+          <t>Confirm with the BOG team whether onboarding subtasks should be in the Run &amp; Sustain queue.</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
@@ -15090,39 +15090,39 @@
           <t>F-26</t>
         </is>
       </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>Needs Verification</t>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Potential Issue</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Transitions - Transition Kickoff Tasks (+SubTask)</t>
+          <t>Set OM and SM overdue tasks to Deferred (1795953061) + all 7 (+SubTask)</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>Action #1 subtasks</t>
+          <t>Parent tasks owned by OM/SM team members</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>Subtask due dates: the parent is due in 7 business days at 8:00 AM (VERIFIED, matches 21/21 records), but its subtasks are due 1-7 business days after creation (e.g. subtask 1 in 1 bd, subtask 7 in 5 bd, subtask 17 in 7 bd). The action panel lists only the subtask titles, so where these per-subtask due dates and the "no owner" setting come from is not visible.</t>
+          <t>A different workflow can defer Transitions tasks automatically. "Set OM and SM overdue tasks to Deferred" (readable, ON) sets Status = DEFERRED on overdue, not-completed tasks whose owner team is 58458611 or 58458777. The 4 DEFERRED Transitions tasks are all "Transition | LAUNCH READINESS | Subtask - Hunter" parents (owner Hunter Stoner) (INFERENCE: deferred by this workflow; the team names/members could not be read - scope settings.users.teams.read missing). Subtasks have no owner, so this workflow can never act on them.</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>Action 1 panel (Due date 7, business days only); subtask due dates in records (Task &amp; Subtask Logic).</t>
+          <t>Config of workflow 1795953061 (VERIFIED: enrollment = hs_task_is_overdue true AND hubspot_team_id in [58458611, 58458777] AND status not Completed; action 1 sets hs_task_status = DEFERRED). Task records: 4 DEFERRED parents, all owner 80038421.</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>Needed to confirm F-02 (subtasks without owners) is a setting, not a side effect.</t>
+          <t>A deferred Launch Readiness parent drops out of overdue views while its subtask (2. Finalize BOG candidates) can still be open.</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>Click one subtask inside Action 1 and screenshot its settings (owner and due date).</t>
+          <t>Confirm which users are in teams 58458611 / 58458777 and whether Transitions tasks should be excluded from auto-deferral.</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
@@ -15137,39 +15137,39 @@
           <t>F-27</t>
         </is>
       </c>
-      <c r="B28" s="10" t="inlineStr">
-        <is>
-          <t>No Issue Found</t>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>All 7 (+SubTask)</t>
+          <t>Transitions - Transition Kickoff Tasks (+SubTask)</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>Enrollment</t>
+          <t>Action #1 associations</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>Every ticket whose latest entry into a stage is after the matching (+SubTask) workflow went live got exactly one enrollment, with the single exception in F-07 (based on the latest "Date entered" value per stage; earlier entries are overwritten). No delays between task actions (all tasks of an enrollment created within ~1-85 seconds).</t>
+          <t>The contact association never adds anyone. Action 1 is set to associate "associated contacts" with label "Transition" (VERIFIED screenshot), but none of the 420 Kickoff tasks is linked to a contact. All 21 Kickoff tickets do have contacts, but none of those ticket-contact associations carries the "Transition" label (they are all unlabelled).</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>Enrollment evidence sheet; stage-entry dates of all 262 Onboarding Pipeline tickets.</t>
+          <t>Action 1 panel: "Associated contacts - Associate Transition". Ticket-&gt;contact association labels on the 21 Kickoff tickets: 21 unlabelled, 0 "Transition" (label typeId 72 exists). Task-&gt;contact associations: 0/420.</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>Task creation itself is reliable once a ticket reaches a stage.</t>
+          <t>Kickoff tasks never appear on the customer contact's record, although the setting suggests they should.</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>Decide whether to label the main customer contact "Transition" on each ticket, or change the action to all associated contacts.</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr">
@@ -15184,39 +15184,39 @@
           <t>F-28</t>
         </is>
       </c>
-      <c r="B29" s="8" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Needs Verification</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Set task queue (1677143128) + Kickoff (+SubTask) + Launch Readiness (+SubTask)</t>
+          <t>Transitions - Transition Kickoff Tasks (+SubTask)</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>Kickoff #1 subtask 9; Launch Readiness #2 subtask 2</t>
+          <t>Action #1 subtasks</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>A different workflow moves two Transitions subtasks into the "BOG - Run and Sustain" task queue. "Set task queue" (readable, ON) enrolls every newly created task and, if the title contains "BOG", sets Queue = 9999918 (its "BOG - Run and Sustain" branch). "9. Submit BOG request in HubSpot to Hunter" (21/21) and "2. Finalize BOG candidates, paperwork, details in Hubspot" (20/20) are in that queue; no other Transitions task is in any queue.</t>
+          <t>Action 1 is set to associate the task with all associated companies (VERIFIED screenshot). The parent got the company in 20/21 enrollments, but in the 4 earliest enrollments (2026-08-24 to 08-27) 13-14 of its 14 subtasks got no company, while the parent did. From 2026-08-28 subtasks get the company too. (The 2026-09-01 ticket had no company at all.)</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>Config of workflow 1677143128 (VERIFIED: list branch "BOG - Run and Sustain" -&gt; action 3 sets hs_queue_membership_ids = 9999918). Task records: hs_queue_membership_ids = 9999918 on exactly those 41 subtasks.</t>
+          <t>Task-&gt;company associations of Kickoff Action #1 subtasks vs. their parent, by enrollment date.</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>Onboarding subtasks with no owner show up in a Run &amp; Sustain queue. That may be how Hunter's team finds them, or it may be unintended.</t>
+          <t>Suggests subtasks did not inherit the parent's associations until about 2026-08-28 (a HubSpot or workflow change). Older subtasks do not show on the company record.</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>Confirm with the BOG team whether onboarding subtasks should be in the Run &amp; Sustain queue.</t>
+          <t>No action needed if the current behaviour is right; optionally add the company to the ~70 older subtasks.</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
@@ -15231,39 +15231,39 @@
           <t>F-29</t>
         </is>
       </c>
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>Potential Issue</t>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Needs Verification</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Set OM and SM overdue tasks to Deferred (1795953061) + all 7 (+SubTask)</t>
+          <t>Transitions - Transition Kickoff Tasks (+SubTask)</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>Parent tasks owned by OM/SM team members</t>
+          <t>Action #1 subtasks</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>A different workflow can defer Transitions tasks automatically. "Set OM and SM overdue tasks to Deferred" (readable, ON) sets Status = DEFERRED on overdue, not-completed tasks whose owner team is 58458611 or 58458777. The 4 DEFERRED Transitions tasks are all "Transition | LAUNCH READINESS | Subtask - Hunter" parents (owner Hunter Stoner) (INFERENCE: deferred by this workflow; the team names/members could not be read - scope settings.users.teams.read missing). Subtasks have no owner, so this workflow can never act on them.</t>
+          <t>Subtask due dates: the parent is due in 7 business days at 8:00 AM (VERIFIED, matches 21/21 records), but its subtasks are due 1-7 business days after creation (e.g. subtask 1 in 1 bd, subtask 7 in 5 bd, subtask 17 in 7 bd). The action panel lists only the subtask titles, so where these per-subtask due dates and the "no owner" setting come from is not visible.</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>Config of workflow 1795953061 (VERIFIED: enrollment = hs_task_is_overdue true AND hubspot_team_id in [58458611, 58458777] AND status not Completed; action 1 sets hs_task_status = DEFERRED). Task records: 4 DEFERRED parents, all owner 80038421.</t>
+          <t>Action 1 panel (Due date 7, business days only); subtask due dates in records (Task &amp; Subtask Logic).</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>A deferred Launch Readiness parent drops out of overdue views while its subtask (2. Finalize BOG candidates) can still be open.</t>
+          <t>Needed to confirm F-02 (subtasks without owners) is a setting, not a side effect.</t>
         </is>
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>Confirm which users are in teams 58458611 / 58458777 and whether Transitions tasks should be excluded from auto-deferral.</t>
+          <t>Click one subtask inside Action 1 and screenshot its settings (owner and due date).</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">

</xml_diff>